<commit_message>
feat: subject library stack, dev:with-api single-window, DWD/DIM and docs
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Source_Data/DIM/全量企业基础维度表.xlsx
+++ b/Source_Data/DIM/全量企业基础维度表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PythonCode\Invoice_Insight_Project\Source_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PythonCode\InvoiceLens\Source_Data\DIM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C90B0B2A-AB13-458F-836E-530FC3B0FEFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC73394B-067D-4159-B00C-80A57045A8AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6048" yWindow="4440" windowWidth="23040" windowHeight="12120" xr2:uid="{16D95BE3-F0A6-4448-AD5A-B59ADB6B0E83}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{16D95BE3-F0A6-4448-AD5A-B59ADB6B0E83}"/>
   </bookViews>
   <sheets>
     <sheet name="全量企业基础维度表" sheetId="1" r:id="rId1"/>
@@ -1083,6 +1083,8 @@
   <cols>
     <col min="1" max="1" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>